<commit_message>
docs: resolve guideline items confirmed by user testing evidence
</commit_message>
<xml_diff>
--- a/phase-a/phase-a-guideline-checklist.xlsx
+++ b/phase-a/phase-a-guideline-checklist.xlsx
@@ -612,7 +612,7 @@
     <row r="12" ht="26.85" customHeight="1" s="17">
       <c r="A12" s="19" t="inlineStr">
         <is>
-          <t>Non verificato — richiede l'accesso autenticato (SPID/CIE/account) che il team non ha potuto testare in questa fase; da verificare nello User Testing con soggetti reali</t>
+          <t>Non verificato — non ispezionabile durante l'expert review (richiedeva accesso autenticato) e non coperto dai 3 task specifici dello User Testing preliminare (Documenti 06a/06b); alcune voci sono state risolte dove i test lo permettevano, le restanti richiedono un'ispezione dedicata nelle fasi successive</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="30" customHeight="1" s="17">
       <c r="A3" s="22" t="inlineStr">
         <is>
@@ -1736,12 +1735,12 @@
       </c>
       <c r="D20" s="30" t="inlineStr">
         <is>
-          <t>Non verificato</t>
+          <t>Non conforme</t>
         </is>
       </c>
       <c r="E20" s="27" t="inlineStr">
         <is>
-          <t>Richiede sessione autenticata per verificare interruzione/ripresa task</t>
+          <t>Confermato dal test utente: la sessione di Amina scade dopo un'interruzione di 40s (telefonata) durante T2, costringendola a ripetere l'accesso e perdendo il progresso (Documento 06a, ID-11).</t>
         </is>
       </c>
       <c r="F20" s="30" t="inlineStr">
@@ -1916,7 +1915,7 @@
       </c>
       <c r="E25" s="27" t="inlineStr">
         <is>
-          <t>Non riscontrati link rotti nell'ispezione pubblica, ma copertura limitata alle pagine non autenticate</t>
+          <t>Nessun link rotto riscontrato nei 4 test utente autenticati (booking, disdetta, assistenza), ma la copertura resta parziale: i test hanno coperto solo i 3 task previsti, non un'ispezione sistematica di tutte le sezioni del sito (Documento 06a).</t>
         </is>
       </c>
       <c r="F25" s="30" t="inlineStr">
@@ -2436,12 +2435,12 @@
       </c>
       <c r="D40" s="30" t="inlineStr">
         <is>
-          <t>Non verificato</t>
+          <t>Parzialmente conforme</t>
         </is>
       </c>
       <c r="E40" s="27" t="inlineStr">
         <is>
-          <t>Richiede completamento di una prenotazione autenticata per verifica diretta</t>
+          <t>Confermato dal test utente: Elena e Amina completano la disdetta (T2) e ricevono un messaggio di conferma, ma generico ('operazione eseguita'), senza riepilogo verificabile (Documento 06a, ID-09).</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
@@ -3636,12 +3635,12 @@
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Non verificato</t>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="G74" s="27" t="inlineStr">
         <is>
-          <t>Elemento non ispezionabile in profondità senza un account attivo; da verificare nello User Testing</t>
+          <t>Confermato dal test utente: tutti e 4 i soggetti usano filtri (specializzazione, città, distanza, disponibilità) in aggiunta alla ricerca testuale (Documento 06b, T1).</t>
         </is>
       </c>
     </row>
@@ -3671,12 +3670,12 @@
       </c>
       <c r="F75" s="30" t="inlineStr">
         <is>
-          <t>Non verificato</t>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="G75" s="27" t="inlineStr">
         <is>
-          <t>Elemento non ispezionabile in profondità senza un account attivo; da verificare nello User Testing</t>
+          <t>Confermato dal test utente: i risultati mostrano informazioni di contesto utili per tutti e 4 i soggetti (prezzo per Renato, foto e mappa per Pina, filtro disponibilità per Elena, filtro distanza per Amina; Documento 06b, T1).</t>
         </is>
       </c>
     </row>
@@ -3706,12 +3705,12 @@
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Non verificato</t>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="G76" s="27" t="inlineStr">
         <is>
-          <t>Tolleranza a errori di battitura non testata direttamente in questa fase</t>
+          <t>Confermato dal test utente: durante il test di Pina (T1) il suggerimento automatico corregge un errore di digitazione (Documento 06b).</t>
         </is>
       </c>
     </row>
@@ -3836,22 +3835,22 @@
       </c>
       <c r="D80" s="30" t="inlineStr">
         <is>
-          <t>Non verificato</t>
+          <t>Non conforme</t>
         </is>
       </c>
       <c r="E80" s="27" t="inlineStr">
         <is>
-          <t>Elemento non ispezionabile senza credenziali SPID/CIE reali; da verificare nello User Testing</t>
+          <t>Confermato dal test utente (T3, 4 soggetti): Pina non completa il task, Elena e Amina trovano solo il canale telefonico ma cercavano un canale scritto compatibile con i loro vincoli (Documento 06a, ID-12).</t>
         </is>
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Non verificato</t>
+          <t>Conforme</t>
         </is>
       </c>
       <c r="G80" s="27" t="inlineStr">
         <is>
-          <t>Elemento non ispezionabile in profondità senza un account attivo; da verificare nello User Testing</t>
+          <t>Confermato dal test utente: tutti e 4 i soggetti trovano rapidamente un canale di contatto (telefono o messaggistica) su T3, con successo pieno o quasi (Documento 06b).</t>
         </is>
       </c>
     </row>
@@ -3906,12 +3905,12 @@
       </c>
       <c r="D82" s="30" t="inlineStr">
         <is>
-          <t>Non verificato</t>
+          <t>Non conforme</t>
         </is>
       </c>
       <c r="E82" s="27" t="inlineStr">
         <is>
-          <t>Elemento non ispezionabile senza credenziali SPID/CIE reali; da verificare nello User Testing</t>
+          <t>Confermato dal test utente: Pina (T1) sbaglia la password demo e non riesce a interpretare il messaggio di errore ('Non so cosa ho sbagliato'), Documento 06a.</t>
         </is>
       </c>
       <c r="F82" s="30" t="inlineStr">
@@ -3941,12 +3940,12 @@
       </c>
       <c r="D83" s="30" t="inlineStr">
         <is>
-          <t>Non verificato</t>
+          <t>Non conforme</t>
         </is>
       </c>
       <c r="E83" s="27" t="inlineStr">
         <is>
-          <t>Elemento non ispezionabile senza credenziali SPID/CIE reali; da verificare nello User Testing</t>
+          <t>Confermato dal test utente: Renato e Pina (T2) individuano il pulsante corretto ma non lo premono per timore di un'azione irreversibile, in assenza di conferma/rassicurazione esplicita (Documento 06a, ID-08).</t>
         </is>
       </c>
       <c r="F83" s="30" t="inlineStr">
@@ -4046,12 +4045,12 @@
       </c>
       <c r="D86" s="30" t="inlineStr">
         <is>
-          <t>Non verificato</t>
+          <t>Parzialmente conforme</t>
         </is>
       </c>
       <c r="E86" s="27" t="inlineStr">
         <is>
-          <t>Elemento non ispezionabile senza credenziali SPID/CIE reali; da verificare nello User Testing</t>
+          <t>Confermato dal test utente: feedback presente dopo le azioni (messaggio di errore al login, conferma dopo disdetta) ma non sempre interpretabile (Pina, Documento 06a).</t>
         </is>
       </c>
       <c r="F86" s="29" t="inlineStr">

</xml_diff>